<commit_message>
[Fix] Dead/Jump → Walk 트랜지션 Condition 추가, 이벤트 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/CBAEvent.xlsx
+++ b/JsonConverter/ExcelFiles/CBAEvent.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\CBA\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AAE6493-6A2C-48D2-B9AE-8CD32C127743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85652FE4-E954-4A6F-8CF1-11845CF674E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="74">
   <si>
     <t>string</t>
   </si>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>돌아서 안전하게 가자.</t>
-  </si>
-  <si>
-    <t>돌아가다 길을 잃었다..</t>
   </si>
   <si>
     <t>event_2</t>
@@ -309,11 +306,270 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>현명한 선택. \n우리 엄마가 길에 있는 건 먹지 말랬어!</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>나무가 저리 가라며 쫓아냈다… \n너무해 엉엉</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>돌아가다 길을 잃었다.. \n나 길치다곰…</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>현명한 선택이었다곰. \n우리 엄마가 길에 있는 건 먹지 말랬어!</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>event_4</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>수상한 버섯</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>알록달록한 버섯을 발견했다.\n먹음직스럽기도 하고 수상하기도 하다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>일단 입에 댄다. 난 곰이니까!</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>건강한 버섯이었다. 난 버섯을 좋아해! \n홍홍~</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>배가 꼬르륵 거리며 복통이 느껴진다…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>헉…</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>뭘 먹은거지?ㅠㅠ</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>그 정도로 멍청하진 않다곰! 냄새만 맡는다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>흥</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>냄새만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>맡고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>현명하게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>지나쳤다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.\n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>나를 뭐로 보는거야?</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>재채기가 멈추지 않는다...\n푸엑취!우엑취!!!\n훌쩍…</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>event_5</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>길 잃은 아기새</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>나무 아래 아기새 한 마리가 떨어져 있다.\n가엾게 삐약삐약 울고 있다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>둥지에 올려준다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>아기새가 안전하게 둥지로 돌아갔다.\n기분이 따뜻해졌다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>나무에서 떨어졌다. 엉덩이가 아프다.\n아기새가 한심하게 쳐다본다ㅠㅠ</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>마음은 무겁고 발걸음은 가볍다. (이거 맞지?)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>죄책감에 발이 무겁다…\n아기새야 미안해…</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>event_6</t>
+  </si>
+  <si>
+    <t>돼지머리가 왜 여기에</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>입에 전재산 만 원을 물려주고 떠난다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>아무 일도 일어나지 않았다. 내 돈…</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>길 한복판에 잘린 돼지머리를 발견했다.\n이게 뭐람?</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>발로 찬다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>돼지머리가 뻥 하고 날아가 사라졌다. 스트레스가 풀렸다.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>빗나가서 발목을 삐었다… 힘만 썼다…</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>어미새가 근처에 있을거라 믿고 지나친다</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>갑자기 돼지머리가 말을 한다:\n이딴 코딱지를 누굴 줘?\n도로 가져가! 투테퉤!!</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -321,7 +577,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="16">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -395,6 +651,40 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="굴림"/>
       <family val="2"/>
       <charset val="129"/>
     </font>
@@ -521,7 +811,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -587,6 +877,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -817,7 +1115,7 @@
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" style="3"/>
+    <col min="2" max="2" width="13.42578125" style="3" customWidth="1"/>
     <col min="3" max="3" width="33.7109375" style="3" customWidth="1"/>
     <col min="4" max="4" width="22.42578125" style="3" customWidth="1"/>
     <col min="5" max="5" width="14.140625" style="22" customWidth="1"/>
@@ -848,18 +1146,18 @@
       <c r="E1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="34" t="s">
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="33"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="37"/>
     </row>
     <row r="2" spans="1:15" ht="12.75">
       <c r="A2" s="1" t="s">
@@ -951,7 +1249,7 @@
         <v>21</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="21"/>
@@ -959,10 +1257,10 @@
         <v>22</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I4" s="21">
         <v>60</v>
@@ -971,10 +1269,10 @@
         <v>23</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L4" s="23" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="M4" s="5">
         <v>80</v>
@@ -984,34 +1282,34 @@
     </row>
     <row r="5" spans="1:15" ht="15.75" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="C5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>27</v>
-      </c>
       <c r="G5" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="I5" s="22">
         <v>50</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L5" s="23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M5" s="5">
         <v>50</v>
@@ -1021,34 +1319,34 @@
     </row>
     <row r="6" spans="1:15" ht="15.75" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="C6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="F6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="19" t="s">
-        <v>32</v>
-      </c>
       <c r="G6" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="I6" s="22">
         <v>20</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L6" s="23" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M6" s="5">
         <v>80</v>
@@ -1057,26 +1355,113 @@
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="A7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="22">
+        <v>50</v>
+      </c>
+      <c r="J7" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="K7" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="M7" s="5">
+        <v>60</v>
+      </c>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
     </row>
     <row r="8" spans="1:15" ht="15.75" customHeight="1">
-      <c r="A8" s="4"/>
-      <c r="B8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
+      <c r="A8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="22">
+        <v>65</v>
+      </c>
+      <c r="J8" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="K8" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="L8" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="M8" s="5">
+        <v>90</v>
+      </c>
       <c r="N8" s="5"/>
       <c r="O8" s="5"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" customHeight="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
+      <c r="A9" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" s="22">
+        <v>70</v>
+      </c>
+      <c r="J9" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="L9" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="M9" s="5">
+        <v>70</v>
+      </c>
       <c r="N9" s="5"/>
       <c r="O9" s="5"/>
     </row>
@@ -1183,7 +1568,7 @@
     </row>
     <row r="16" spans="1:15" ht="15.75" customHeight="1">
       <c r="A16" s="4"/>
-      <c r="C16" s="16"/>
+      <c r="C16" s="31"/>
       <c r="D16" s="6"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
@@ -1195,7 +1580,7 @@
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1">
       <c r="A17" s="4"/>
-      <c r="C17" s="16"/>
+      <c r="C17" s="31"/>
       <c r="D17" s="6"/>
       <c r="E17" s="21"/>
       <c r="F17" s="21"/>

</xml_diff>